<commit_message>
Kaltpruefung Block 2: Metadaten, interne Verweise, Abhaengigkeiten, Normtext-Chunks
- 18: PDF-Autor Wolfgang Bossle
- 19: Anlagenbuchhaltung A1/A2 Muster Baeckerei GmbH, Fiktiver Musterfall
- 20: interne Verweise (Grundsatz-Nummern, PROJECT.md, docs/, .claude,
  CCA, Kandidat) entfernt; Paketname ki-jahresabschluss-hgb
- 21: Zaehlung der Registerauszuege gestrichen
- 22: Mapping-Hinweis auf Musterkonten beschraenkt
- 23: pyproject 1.0.0, CITATION date-released
- 28: python-docx statt pdfplumber, uv.lock neu
- 14: chunks.json IDs und Titel aus absatz, geltungsbereich entfernt
- 15: Section grundanteil_hinweis gestrichen
- 32: taxonomy_complete_gmbh.json entfernt, Kommentare korrigiert
- 33: render_pdf_demo.py schreibt nach output/local/, --release fuer das
  eingecheckte PDF

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/baeckerei_2025/Anlagenbuchhaltung.xlsx
+++ b/data/baeckerei_2025/Anlagenbuchhaltung.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anlagenbuchhaltung" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hinweise" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Anlagenbuchhaltung" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hinweise" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,14 +444,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bäckerei Hoffmann GmbH  |  Anlagenbuchhaltung  |  Geschäftsjahr 01.01.2025 – 31.12.2025</t>
+          <t>Muster Bäckerei GmbH  |  Anlagenbuchhaltung  |  Geschäftsjahr 01.01.2025 – 31.12.2025</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fiktiver Testfall – 8_AI_Accounting Showcase  |  Alle Beträge in EUR</t>
+          <t>Fiktiver Musterfall  |  Alle Beträge in EUR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kaltpruefung Befund 10: Zugang 0441 mit Lieferung 28.12.2025, betriebsbereit ab 01/2026
Hinweiszeile im Blatt Hinweise; Zahlen unveraendert. Ausweisfrage Anlagen im Bau bewusst offen.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dfab1A2oWEqthFM5tHPSti
</commit_message>
<xml_diff>
--- a/data/baeckerei_2025/Anlagenbuchhaltung.xlsx
+++ b/data/baeckerei_2025/Anlagenbuchhaltung.xlsx
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -977,6 +977,23 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Technische Anlagen und Maschinen (Konto 0441)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Zugang Ofen 150.000 EUR: Lieferung am 28.12.2025, betriebsbereit ab Januar 2026. Planmäßige Abschreibung ab 2026, im Geschäftsjahr 2025 daher keine AfA.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>